<commit_message>
Islande izslēgta no reitingiem, labāki negatīvo vērtību uzraksti
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TofK8gUjxHJeGVCYw9TpEQ
</commit_message>
<xml_diff>
--- a/docs/dati/aizsardzibas_izdevumi.xlsx
+++ b/docs/dati/aizsardzibas_izdevumi.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lasi mani" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="% no IKP" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Uz 1 iedzīvotāju (USD)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Reālie izdevumi (milj. USD)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="% no valdības izdevumiem" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Eurostat % no IKP" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Periodu vidējie" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Reģionu vidējie" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Korelācija" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lasi mani" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="% no IKP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uz 1 iedzīvotāju (USD)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reālie izdevumi (milj. USD)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="% no valdības izdevumiem" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eurostat % no IKP" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Periodu vidējie" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reģionu vidējie" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Korelācija" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20149,7 +20149,7 @@
         <v>1.16</v>
       </c>
       <c r="C5" t="n">
-        <v>1.24</v>
+        <v>1.56</v>
       </c>
       <c r="D5" t="n">
         <v>1.71</v>
@@ -20181,7 +20181,7 @@
         <v>1.31</v>
       </c>
       <c r="C6" t="n">
-        <v>1.22</v>
+        <v>1.52</v>
       </c>
       <c r="D6" t="n">
         <v>1.76</v>
@@ -20213,7 +20213,7 @@
         <v>1.51</v>
       </c>
       <c r="C7" t="n">
-        <v>1.27</v>
+        <v>1.59</v>
       </c>
       <c r="D7" t="n">
         <v>1.77</v>
@@ -20245,7 +20245,7 @@
         <v>1.51</v>
       </c>
       <c r="C8" t="n">
-        <v>1.29</v>
+        <v>1.62</v>
       </c>
       <c r="D8" t="n">
         <v>1.82</v>
@@ -20277,7 +20277,7 @@
         <v>1.51</v>
       </c>
       <c r="C9" t="n">
-        <v>1.23</v>
+        <v>1.54</v>
       </c>
       <c r="D9" t="n">
         <v>1.67</v>
@@ -20309,7 +20309,7 @@
         <v>1.43</v>
       </c>
       <c r="C10" t="n">
-        <v>1.15</v>
+        <v>1.44</v>
       </c>
       <c r="D10" t="n">
         <v>1.7</v>
@@ -20341,7 +20341,7 @@
         <v>1.45</v>
       </c>
       <c r="C11" t="n">
-        <v>1.12</v>
+        <v>1.4</v>
       </c>
       <c r="D11" t="n">
         <v>1.57</v>
@@ -20373,7 +20373,7 @@
         <v>1.47</v>
       </c>
       <c r="C12" t="n">
-        <v>1.07</v>
+        <v>1.34</v>
       </c>
       <c r="D12" t="n">
         <v>1.54</v>
@@ -20405,7 +20405,7 @@
         <v>1.53</v>
       </c>
       <c r="C13" t="n">
-        <v>1.06</v>
+        <v>1.32</v>
       </c>
       <c r="D13" t="n">
         <v>1.41</v>
@@ -20437,7 +20437,7 @@
         <v>1.43</v>
       </c>
       <c r="C14" t="n">
-        <v>1.13</v>
+        <v>1.42</v>
       </c>
       <c r="D14" t="n">
         <v>1.44</v>
@@ -20469,7 +20469,7 @@
         <v>1.23</v>
       </c>
       <c r="C15" t="n">
-        <v>1.12</v>
+        <v>1.4</v>
       </c>
       <c r="D15" t="n">
         <v>1.32</v>
@@ -20501,7 +20501,7 @@
         <v>1.19</v>
       </c>
       <c r="C16" t="n">
-        <v>1.07</v>
+        <v>1.34</v>
       </c>
       <c r="D16" t="n">
         <v>1.24</v>
@@ -20533,7 +20533,7 @@
         <v>1.2</v>
       </c>
       <c r="C17" t="n">
-        <v>1.08</v>
+        <v>1.35</v>
       </c>
       <c r="D17" t="n">
         <v>1.24</v>
@@ -20565,7 +20565,7 @@
         <v>1.21</v>
       </c>
       <c r="C18" t="n">
-        <v>1.06</v>
+        <v>1.32</v>
       </c>
       <c r="D18" t="n">
         <v>1.18</v>
@@ -20597,7 +20597,7 @@
         <v>1.25</v>
       </c>
       <c r="C19" t="n">
-        <v>1.04</v>
+        <v>1.3</v>
       </c>
       <c r="D19" t="n">
         <v>1.18</v>
@@ -20629,7 +20629,7 @@
         <v>1.4</v>
       </c>
       <c r="C20" t="n">
-        <v>1.03</v>
+        <v>1.29</v>
       </c>
       <c r="D20" t="n">
         <v>1.27</v>
@@ -20661,7 +20661,7 @@
         <v>1.67</v>
       </c>
       <c r="C21" t="n">
-        <v>1.05</v>
+        <v>1.31</v>
       </c>
       <c r="D21" t="n">
         <v>1.26</v>
@@ -20693,7 +20693,7 @@
         <v>1.78</v>
       </c>
       <c r="C22" t="n">
-        <v>1.05</v>
+        <v>1.31</v>
       </c>
       <c r="D22" t="n">
         <v>1.28</v>
@@ -20725,7 +20725,7 @@
         <v>2.02</v>
       </c>
       <c r="C23" t="n">
-        <v>1.08</v>
+        <v>1.35</v>
       </c>
       <c r="D23" t="n">
         <v>1.33</v>
@@ -20757,7 +20757,7 @@
         <v>2.02</v>
       </c>
       <c r="C24" t="n">
-        <v>1.12</v>
+        <v>1.4</v>
       </c>
       <c r="D24" t="n">
         <v>1.54</v>
@@ -20789,7 +20789,7 @@
         <v>2.18</v>
       </c>
       <c r="C25" t="n">
-        <v>1.19</v>
+        <v>1.48</v>
       </c>
       <c r="D25" t="n">
         <v>1.78</v>
@@ -20821,7 +20821,7 @@
         <v>2.04</v>
       </c>
       <c r="C26" t="n">
-        <v>1.1</v>
+        <v>1.37</v>
       </c>
       <c r="D26" t="n">
         <v>1.63</v>
@@ -20853,7 +20853,7 @@
         <v>2.32</v>
       </c>
       <c r="C27" t="n">
-        <v>1.15</v>
+        <v>1.44</v>
       </c>
       <c r="D27" t="n">
         <v>1.78</v>
@@ -20885,7 +20885,7 @@
         <v>2.92</v>
       </c>
       <c r="C28" t="n">
-        <v>1.47</v>
+        <v>1.84</v>
       </c>
       <c r="D28" t="n">
         <v>2.09</v>
@@ -20917,7 +20917,7 @@
         <v>3.25</v>
       </c>
       <c r="C29" t="n">
-        <v>1.73</v>
+        <v>2.17</v>
       </c>
       <c r="D29" t="n">
         <v>2.43</v>
@@ -20949,7 +20949,7 @@
         <v>3.35</v>
       </c>
       <c r="C30" t="n">
-        <v>2.31</v>
+        <v>2.89</v>
       </c>
       <c r="D30" t="n">
         <v>2.6</v>
@@ -20984,7 +20984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -20996,7 +20996,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Aizsardzības izdevumi un IKP izaugsme (Pīrsona r = -0,14)</t>
+          <t>Aizsardzības izdevumi un IKP izaugsme (Pīrsona r = -0,15)</t>
         </is>
       </c>
     </row>
@@ -21230,25 +21230,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Islande</t>
+          <t>Itālija</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ziemeļvalstis</t>
+          <t>Dienvideiropa</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1.51</v>
       </c>
       <c r="D16" t="n">
-        <v>2.75</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Itālija</t>
+          <t>Kipra</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -21257,34 +21257,34 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.51</v>
+        <v>1.84</v>
       </c>
       <c r="D17" t="n">
-        <v>0.57</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Kipra</t>
+          <t>Latvija</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Dienvideiropa</t>
+          <t>Baltijas valstis</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.84</v>
+        <v>1.74</v>
       </c>
       <c r="D18" t="n">
-        <v>3.25</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Latvija</t>
+          <t>Lietuva</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -21293,178 +21293,178 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.74</v>
+        <v>1.53</v>
       </c>
       <c r="D19" t="n">
-        <v>3.26</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Lietuva</t>
+          <t>Luksemburga</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Baltijas valstis</t>
+          <t>Rietumeiropa</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1.53</v>
+        <v>0.49</v>
       </c>
       <c r="D20" t="n">
-        <v>3.92</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Luksemburga</t>
+          <t>Malta</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Rietumeiropa</t>
+          <t>Dienvideiropa</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.49</v>
+        <v>0.55</v>
       </c>
       <c r="D21" t="n">
-        <v>2.49</v>
+        <v>5.21</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Malta</t>
+          <t>Melnkalne</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dienvideiropa</t>
+          <t>Dienvidaustrumeiropa</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.55</v>
+        <v>1.7</v>
       </c>
       <c r="D22" t="n">
-        <v>5.21</v>
+        <v>3.07</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Melnkalne</t>
+          <t>Moldova</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dienvidaustrumeiropa</t>
+          <t>Austrumeiropa</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
       <c r="D23" t="n">
-        <v>3.07</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Moldova</t>
+          <t>Norvēģija</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Austrumeiropa</t>
+          <t>Ziemeļvalstis</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.4</v>
+        <v>1.72</v>
       </c>
       <c r="D24" t="n">
-        <v>3.63</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Norvēģija</t>
+          <t>Nīderlande</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ziemeļvalstis</t>
+          <t>Rietumeiropa</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.72</v>
+        <v>1.37</v>
       </c>
       <c r="D25" t="n">
-        <v>1.84</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Nīderlande</t>
+          <t>Polija</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rietumeiropa</t>
+          <t>Centrāleiropa</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1.37</v>
+        <v>2.15</v>
       </c>
       <c r="D26" t="n">
-        <v>1.62</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Polija</t>
+          <t>Portugāle</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Centrāleiropa</t>
+          <t>Dienvideiropa</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2.15</v>
+        <v>1.5</v>
       </c>
       <c r="D27" t="n">
-        <v>3.64</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Portugāle</t>
+          <t>Rumānija</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dienvideiropa</t>
+          <t>Dienvidaustrumeiropa</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1.5</v>
+        <v>1.75</v>
       </c>
       <c r="D28" t="n">
-        <v>1.13</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rumānija</t>
+          <t>Serbija</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -21473,214 +21473,214 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1.75</v>
+        <v>2.4</v>
       </c>
       <c r="D29" t="n">
-        <v>3.48</v>
+        <v>3.29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Serbija</t>
+          <t>Slovākija</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dienvidaustrumeiropa</t>
+          <t>Centrāleiropa</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2.4</v>
+        <v>1.5</v>
       </c>
       <c r="D30" t="n">
-        <v>3.29</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Slovākija</t>
+          <t>Slovēnija</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Centrāleiropa</t>
+          <t>Dienvidaustrumeiropa</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1.5</v>
+        <v>1.28</v>
       </c>
       <c r="D31" t="n">
-        <v>3.22</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Slovēnija</t>
+          <t>Somija</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dienvidaustrumeiropa</t>
+          <t>Ziemeļvalstis</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1.28</v>
+        <v>1.51</v>
       </c>
       <c r="D32" t="n">
-        <v>2.36</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Somija</t>
+          <t>Spānija</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Ziemeļvalstis</t>
+          <t>Dienvideiropa</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.51</v>
+        <v>1.4</v>
       </c>
       <c r="D33" t="n">
-        <v>1.25</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Spānija</t>
+          <t>Turcija</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dienvideiropa</t>
+          <t>Dienvidaustrumeiropa</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1.4</v>
+        <v>2.33</v>
       </c>
       <c r="D34" t="n">
-        <v>1.84</v>
+        <v>5.05</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Turcija</t>
+          <t>Ungārija</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dienvidaustrumeiropa</t>
+          <t>Centrāleiropa</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2.33</v>
+        <v>1.36</v>
       </c>
       <c r="D35" t="n">
-        <v>5.05</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ungārija</t>
+          <t>Vācija</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Centrāleiropa</t>
+          <t>Rietumeiropa</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1.36</v>
+        <v>1.3</v>
       </c>
       <c r="D36" t="n">
-        <v>2.36</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Vācija</t>
+          <t>Ziemeļmaķedonija</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Rietumeiropa</t>
+          <t>Dienvidaustrumeiropa</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1.3</v>
+        <v>1.74</v>
       </c>
       <c r="D37" t="n">
-        <v>1.08</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ziemeļmaķedonija</t>
+          <t>Zviedrija</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dienvidaustrumeiropa</t>
+          <t>Ziemeļvalstis</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.74</v>
+        <v>1.35</v>
       </c>
       <c r="D38" t="n">
-        <v>2.67</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Zviedrija</t>
+          <t>Čehija</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ziemeļvalstis</t>
+          <t>Centrāleiropa</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1.35</v>
+        <v>1.37</v>
       </c>
       <c r="D39" t="n">
-        <v>1.98</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Čehija</t>
+          <t>Īrija</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Centrāleiropa</t>
+          <t>Rietumeiropa</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1.37</v>
+        <v>0.44</v>
       </c>
       <c r="D40" t="n">
-        <v>2.43</v>
+        <v>5.51</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Īrija</t>
+          <t>Šveice</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -21689,27 +21689,9 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.44</v>
+        <v>0.75</v>
       </c>
       <c r="D41" t="n">
-        <v>5.51</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Šveice</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Rietumeiropa</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D42" t="n">
         <v>1.92</v>
       </c>
     </row>

</xml_diff>